<commit_message>
don't put bw on blank form!
</commit_message>
<xml_diff>
--- a/owlcms/src/main/resources/templates/weighin/WeighInForm-LETTER.xlsx
+++ b/owlcms/src/main/resources/templates/weighin/WeighInForm-LETTER.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lamyj\git\owlcms4\owlcms\src\main\resources\templates\weighin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91BC8F16-658A-4A29-B8E8-8545BB7DE093}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E225AA8-7634-4552-9B56-1A1292ECD058}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4275" yWindow="1725" windowWidth="21600" windowHeight="11295" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="1815" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Weigh-in" sheetId="1" r:id="rId1"/>
@@ -54,7 +54,7 @@
     <definedName name="TAS">'Weigh-in'!#REF!</definedName>
     <definedName name="tirage">'Weigh-in'!#REF!</definedName>
   </definedNames>
-  <calcPr calcId="0" iterateDelta="1E-4"/>
+  <calcPr calcId="0"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="36">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>${t.get("Competition.competitionName")} :</t>
   </si>
@@ -142,9 +142,6 @@
   </si>
   <si>
     <t>${l.lastName}, ${l.firstName}</t>
-  </si>
-  <si>
-    <t>${l.bodyWeight}</t>
   </si>
   <si>
     <t>${l.club}</t>
@@ -1098,20 +1095,18 @@
       <c r="C14" s="36" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="37" t="s">
+      <c r="D14" s="37"/>
+      <c r="E14" s="38" t="s">
         <v>26</v>
       </c>
-      <c r="E14" s="38" t="s">
+      <c r="F14" s="39" t="s">
         <v>27</v>
       </c>
-      <c r="F14" s="39" t="s">
+      <c r="G14" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="G14" s="40" t="s">
+      <c r="H14" s="1" t="s">
         <v>29</v>
-      </c>
-      <c r="H14" s="1" t="s">
-        <v>30</v>
       </c>
       <c r="I14" s="1"/>
       <c r="J14" s="1"/>
@@ -1120,7 +1115,7 @@
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E15"/>
     </row>
@@ -1130,10 +1125,10 @@
     </row>
     <row r="17" spans="3:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C17" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" s="43" t="s">
         <v>32</v>
-      </c>
-      <c r="D17" s="43" t="s">
-        <v>33</v>
       </c>
       <c r="E17" s="43"/>
       <c r="F17" s="43"/>
@@ -1143,10 +1138,10 @@
     </row>
     <row r="18" spans="3:20" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="C18" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" s="43" t="s">
         <v>34</v>
-      </c>
-      <c r="D18" s="43" t="s">
-        <v>35</v>
       </c>
       <c r="E18" s="43"/>
       <c r="F18" s="43"/>

</xml_diff>